<commit_message>
Update session details and speaker information for Endogineco 2026
- Corrected speaker names and titles in the program schedule, including changing "Helena Nagle" to "Helena Nagy" and "Priscilla Vieira" to "Priscila Vieira."
- Enhanced session descriptions for clarity and consistency across the schedule.
- Updated CSV files for pre-congress courses, ensuring accurate speaker names and session details.
- Improved HTML generation script to better format session information and speaker details in the schedule.
</commit_message>
<xml_diff>
--- a/endogineco2026/pre-congress/programacao-pre-congresso.xlsx
+++ b/endogineco2026/pre-congress/programacao-pre-congresso.xlsx
@@ -9,7 +9,7 @@
     <sheet name="PRÉ CONGRESSO (GERAL) " sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PRÉ CONGRESSO (GERAL) '!$A$1:$C$78</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PRÉ CONGRESSO (GERAL) '!$A$1:$C$79</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
   <si>
     <t xml:space="preserve">PRÉ CONGRESSO ENDOGINECO 2026 </t>
   </si>
@@ -279,92 +279,107 @@
     <t xml:space="preserve">O que há de Novo na Literatura Mundial: As evidências científicas e diretrizes internacionais mais recentes que estão mudando a conduta na endometriose profunda.</t>
   </si>
   <si>
-    <t xml:space="preserve">12:30 - 19:00</t>
+    <t xml:space="preserve">12:00 - 19:00</t>
   </si>
   <si>
     <t xml:space="preserve">FOYER - Curso de Sutura Dry Lab em sutura Endoscópica 
 Coordenação: Guilherme Zanluchi - SP</t>
   </si>
   <si>
-    <t xml:space="preserve">12:30 - 13:00 </t>
+    <t xml:space="preserve">12:00 - 12:30</t>
   </si>
   <si>
     <t xml:space="preserve">Regras básicas de posição de agulha e fio - Nomenclatura e sistematização de agulha</t>
   </si>
   <si>
-    <t xml:space="preserve">professor 1</t>
+    <t xml:space="preserve">Helena Nagy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:30 - 13:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teoria do Ponto perfeito e passagem de agulha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sidraiton Melo </t>
   </si>
   <si>
     <t xml:space="preserve">13:00 - 13:30</t>
   </si>
   <si>
-    <t xml:space="preserve">Teoria do Ponto perfeito e passagem de agulha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">professor 2</t>
-  </si>
-  <si>
-    <t>13:30-14:00</t>
-  </si>
-  <si>
     <t xml:space="preserve">Aplicação prática de sutura em videos: Fechamento de cúpula vaginal e miomectomias</t>
   </si>
   <si>
-    <t xml:space="preserve">professor 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14:00 - 15:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estação prática</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14:00-14:30 </t>
+    <t xml:space="preserve">Guilherme Zanluchi - SP </t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:30 - 15:15
+(01 hora e 
+45 minutos) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estação prática
+Monitores: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:30 - 14:05</t>
   </si>
   <si>
     <t xml:space="preserve">Sistematização de 1 grau e acordar as mãos</t>
   </si>
   <si>
-    <t>14:30-15:00</t>
+    <t xml:space="preserve">14:05 - 14:40</t>
   </si>
   <si>
     <t xml:space="preserve">Sistematizaçoes e Cruz de verificaçao</t>
   </si>
   <si>
-    <t xml:space="preserve">15:00 -15:30</t>
+    <t xml:space="preserve">14:40 - 15:15</t>
   </si>
   <si>
     <t xml:space="preserve">O Ponto Perfeito</t>
   </si>
   <si>
-    <t xml:space="preserve">16:00 - 16:30</t>
+    <t xml:space="preserve">15:15 - 15:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:45 - 16:15</t>
   </si>
   <si>
     <t xml:space="preserve">Teoria dos nós: Nó quadrado e semi-chaves</t>
   </si>
   <si>
-    <t xml:space="preserve">16:30 - 17:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Os nós da minha preferência - Aplicação dos nós em cada tipo de tecido e cirurgia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:30 - 19:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:30 - 18:00</t>
+    <t xml:space="preserve">16:15 - 16:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segurança dos nós </t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:45 - 17:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os nós da minha preferência - Aplicação dos nós em cada tipo de tecido e cirurgia
+(Triplo / Duplo) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:15 - 19:00
+(01 hora e 
+45 minutos) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:15 - 17:50</t>
   </si>
   <si>
     <t xml:space="preserve">Triplo Duplo - Monomanual e bimanual</t>
   </si>
   <si>
-    <t xml:space="preserve">18:00 - 18:30</t>
+    <t xml:space="preserve">17:50 - 18:25</t>
   </si>
   <si>
     <t xml:space="preserve">Sequência de semi-chaves bloqueantes</t>
   </si>
   <si>
-    <t xml:space="preserve">18:30 - 19:00</t>
+    <t xml:space="preserve">18:25 - 19:00</t>
   </si>
   <si>
     <t xml:space="preserve">Competição - Prêmio </t>
@@ -377,6 +392,7 @@
   <fonts count="9">
     <font>
       <sz val="11.000000"/>
+      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -429,7 +445,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -533,8 +549,14 @@
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="25">
+  <borders count="26">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -836,6 +858,17 @@
       </bottom>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -844,7 +877,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="105">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1135,17 +1168,26 @@
     <xf fontId="4" fillId="18" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="7" fillId="6" borderId="15" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="7" fillId="6" borderId="16" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="7" fillId="6" borderId="17" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf fontId="8" fillId="7" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="10" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="6" borderId="5" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="6" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf fontId="7" fillId="19" borderId="5" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="19" borderId="22" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="19" borderId="25" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1174,7 +1216,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>44450</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1409698" cy="314350"/>
+    <xdr:ext cx="1409699" cy="314350"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="14" name="Imagem 13"/>
@@ -1770,12 +1812,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultColWidth="10.26953125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="10.1796875" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" style="2" width="15.7265625"/>
     <col customWidth="1" min="2" max="2" style="1" width="72.54296875"/>
-    <col customWidth="1" min="3" max="3" style="1" width="29.26953125"/>
-    <col min="4" max="16384" style="1" width="10.26953125"/>
+    <col customWidth="1" min="3" max="3" style="1" width="29.453125"/>
+    <col min="4" max="16384" style="1" width="10.1796875"/>
   </cols>
   <sheetData>
     <row r="1" ht="39.649999999999999" customHeight="1">
@@ -1785,7 +1827,7 @@
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
     </row>
-    <row r="2" s="5" customFormat="1" ht="16.5">
+    <row r="2" s="5" customFormat="1" ht="15.5">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
@@ -2362,7 +2404,7 @@
       </c>
       <c r="D67" s="89"/>
     </row>
-    <row r="68" s="89" customFormat="1" ht="24.75" customHeight="1">
+    <row r="68" s="89" customFormat="1" ht="40" customHeight="1">
       <c r="A68" s="95" t="s">
         <v>95</v>
       </c>
@@ -2379,7 +2421,7 @@
       <c r="B69" s="94" t="s">
         <v>98</v>
       </c>
-      <c r="C69" s="94"/>
+      <c r="C69" s="98"/>
       <c r="D69" s="89"/>
     </row>
     <row r="70" s="89" customFormat="1" ht="24.75" customHeight="1">
@@ -2389,7 +2431,7 @@
       <c r="B70" s="94" t="s">
         <v>100</v>
       </c>
-      <c r="C70" s="94"/>
+      <c r="C70" s="99"/>
       <c r="D70" s="89"/>
     </row>
     <row r="71" s="89" customFormat="1" ht="24.75" customHeight="1">
@@ -2399,14 +2441,14 @@
       <c r="B71" s="94" t="s">
         <v>102</v>
       </c>
-      <c r="C71" s="94"/>
+      <c r="C71" s="100"/>
       <c r="D71" s="89"/>
     </row>
     <row r="72" s="89" customFormat="1" ht="24.75" customHeight="1">
       <c r="A72" s="93" t="s">
-        <v>12</v>
-      </c>
-      <c r="B72" s="98" t="s">
+        <v>103</v>
+      </c>
+      <c r="B72" s="101" t="s">
         <v>13</v>
       </c>
       <c r="C72" s="27"/>
@@ -2414,22 +2456,22 @@
     </row>
     <row r="73" s="89" customFormat="1" ht="24.75" customHeight="1">
       <c r="A73" s="93" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B73" s="94" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C73" s="94" t="s">
         <v>88</v>
       </c>
       <c r="D73" s="89"/>
     </row>
-    <row r="74" s="89" customFormat="1" ht="24.75" customHeight="1">
+    <row r="74" s="89" customFormat="1" ht="24.5" customHeight="1">
       <c r="A74" s="93" t="s">
-        <v>105</v>
-      </c>
-      <c r="B74" s="94" t="s">
         <v>106</v>
+      </c>
+      <c r="B74" s="89" t="s">
+        <v>107</v>
       </c>
       <c r="C74" s="94" t="s">
         <v>91</v>
@@ -2438,54 +2480,58 @@
     </row>
     <row r="75" s="89" customFormat="1" ht="24.75" customHeight="1">
       <c r="A75" s="93" t="s">
-        <v>107</v>
-      </c>
-      <c r="B75" s="86" t="s">
-        <v>96</v>
+        <v>108</v>
+      </c>
+      <c r="B75" s="94" t="s">
+        <v>109</v>
       </c>
       <c r="C75" s="94" t="s">
         <v>94</v>
       </c>
       <c r="D75" s="89"/>
     </row>
-    <row r="76" s="89" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A76" s="93" t="s">
-        <v>108</v>
-      </c>
-      <c r="B76" s="94" t="s">
-        <v>109</v>
-      </c>
-      <c r="C76" s="94"/>
+    <row r="76" s="89" customFormat="1" ht="40" customHeight="1">
+      <c r="A76" s="102" t="s">
+        <v>110</v>
+      </c>
+      <c r="B76" s="103" t="s">
+        <v>96</v>
+      </c>
+      <c r="C76" s="104"/>
       <c r="D76" s="89"/>
     </row>
     <row r="77" s="89" customFormat="1" ht="24.75" customHeight="1">
       <c r="A77" s="93" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B77" s="94" t="s">
-        <v>111</v>
-      </c>
-      <c r="C77" s="94"/>
+        <v>112</v>
+      </c>
+      <c r="C77" s="98"/>
       <c r="D77" s="89"/>
     </row>
     <row r="78" s="89" customFormat="1" ht="24.75" customHeight="1">
       <c r="A78" s="93" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B78" s="94" t="s">
-        <v>113</v>
-      </c>
-      <c r="C78" s="94"/>
+        <v>114</v>
+      </c>
+      <c r="C78" s="99"/>
       <c r="D78" s="89"/>
     </row>
-    <row r="79" s="99" customFormat="1" ht="25" customHeight="1">
-      <c r="A79" s="100"/>
-      <c r="B79" s="101"/>
-      <c r="C79" s="101"/>
-      <c r="D79" s="99"/>
+    <row r="79" s="89" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A79" s="93" t="s">
+        <v>115</v>
+      </c>
+      <c r="B79" s="94" t="s">
+        <v>116</v>
+      </c>
+      <c r="C79" s="100"/>
+      <c r="D79" s="89"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="32">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B10:C10"/>
@@ -2514,7 +2560,10 @@
     <mergeCell ref="B60:C60"/>
     <mergeCell ref="B64:C64"/>
     <mergeCell ref="B68:C68"/>
+    <mergeCell ref="C69:C71"/>
     <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="C77:C79"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157477" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>